<commit_message>
refactor: move lógica do main.py para core/inventario.py e corrige mapeamento de priorização
</commit_message>
<xml_diff>
--- a/data/historico/historico_documentos.xlsx
+++ b/data/historico/historico_documentos.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E186"/>
+  <dimension ref="A1:E216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2185,1743 +2185,1981 @@
       <c r="A104" t="n">
         <v>4034123</v>
       </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>2400002805</t>
-        </is>
+      <c r="B104" t="n">
+        <v>2400002805</v>
       </c>
       <c r="C104" t="n">
         <v>400</v>
       </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D104" t="n">
+        <v>600012400</v>
       </c>
       <c r="E104" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
         <v>4000194</v>
       </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>2500045827</t>
-        </is>
+      <c r="B105" t="n">
+        <v>2500045827</v>
       </c>
       <c r="C105" t="n">
         <v>400</v>
       </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D105" t="n">
+        <v>600012400</v>
       </c>
       <c r="E105" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
         <v>4021439</v>
       </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>2500035963</t>
-        </is>
+      <c r="B106" t="n">
+        <v>2500035963</v>
       </c>
       <c r="C106" t="n">
         <v>400</v>
       </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D106" t="n">
+        <v>600012400</v>
       </c>
       <c r="E106" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
         <v>4000688</v>
       </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>2500045655</t>
-        </is>
+      <c r="B107" t="n">
+        <v>2500045655</v>
       </c>
       <c r="C107" t="n">
         <v>400</v>
       </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D107" t="n">
+        <v>600012400</v>
       </c>
       <c r="E107" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
         <v>4036635</v>
       </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>2500043146</t>
-        </is>
+      <c r="B108" t="n">
+        <v>2500043146</v>
       </c>
       <c r="C108" t="n">
         <v>400</v>
       </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D108" t="n">
+        <v>600012400</v>
       </c>
       <c r="E108" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
         <v>4000194</v>
       </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>2500044511</t>
-        </is>
+      <c r="B109" t="n">
+        <v>2500044511</v>
       </c>
       <c r="C109" t="n">
         <v>400</v>
       </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D109" t="n">
+        <v>600012400</v>
       </c>
       <c r="E109" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
         <v>4042278</v>
       </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>2600016475</t>
-        </is>
+      <c r="B110" t="n">
+        <v>2600016475</v>
       </c>
       <c r="C110" t="n">
         <v>400</v>
       </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D110" t="n">
+        <v>600012400</v>
       </c>
       <c r="E110" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
         <v>4033776</v>
       </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>2600001895</t>
-        </is>
+      <c r="B111" t="n">
+        <v>2600001895</v>
       </c>
       <c r="C111" t="n">
         <v>400</v>
       </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D111" t="n">
+        <v>600012400</v>
       </c>
       <c r="E111" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
         <v>4038921</v>
       </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>2500029182</t>
-        </is>
+      <c r="B112" t="n">
+        <v>2500029182</v>
       </c>
       <c r="C112" t="n">
         <v>400</v>
       </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D112" t="n">
+        <v>600012400</v>
       </c>
       <c r="E112" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
         <v>4038921</v>
       </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>2500041942</t>
-        </is>
+      <c r="B113" t="n">
+        <v>2500041942</v>
       </c>
       <c r="C113" t="n">
         <v>400</v>
       </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D113" t="n">
+        <v>600012400</v>
       </c>
       <c r="E113" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
         <v>4038915</v>
       </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>2500041125</t>
-        </is>
+      <c r="B114" t="n">
+        <v>2500041125</v>
       </c>
       <c r="C114" t="n">
         <v>400</v>
       </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D114" t="n">
+        <v>600012400</v>
       </c>
       <c r="E114" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
         <v>4009062</v>
       </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>2500039537</t>
-        </is>
+      <c r="B115" t="n">
+        <v>2500039537</v>
       </c>
       <c r="C115" t="n">
         <v>400</v>
       </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D115" t="n">
+        <v>600012400</v>
       </c>
       <c r="E115" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
         <v>4038915</v>
       </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>2500020147</t>
-        </is>
+      <c r="B116" t="n">
+        <v>2500020147</v>
       </c>
       <c r="C116" t="n">
         <v>400</v>
       </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D116" t="n">
+        <v>600012400</v>
       </c>
       <c r="E116" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
         <v>4036765</v>
       </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>2600007337</t>
-        </is>
+      <c r="B117" t="n">
+        <v>2600007337</v>
       </c>
       <c r="C117" t="n">
         <v>400</v>
       </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D117" t="n">
+        <v>600012400</v>
       </c>
       <c r="E117" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
         <v>3002286</v>
       </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>2600013791</t>
-        </is>
+      <c r="B118" t="n">
+        <v>2600013791</v>
       </c>
       <c r="C118" t="n">
         <v>400</v>
       </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D118" t="n">
+        <v>600012400</v>
       </c>
       <c r="E118" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
         <v>3000283</v>
       </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>2500043884</t>
-        </is>
+      <c r="B119" t="n">
+        <v>2500043884</v>
       </c>
       <c r="C119" t="n">
         <v>400</v>
       </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D119" t="n">
+        <v>600012400</v>
       </c>
       <c r="E119" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
         <v>3000226</v>
       </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>2400039501</t>
-        </is>
+      <c r="B120" t="n">
+        <v>2400039501</v>
       </c>
       <c r="C120" t="n">
         <v>400</v>
       </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D120" t="n">
+        <v>600012400</v>
       </c>
       <c r="E120" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
         <v>3000308</v>
       </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>2300036125</t>
-        </is>
+      <c r="B121" t="n">
+        <v>2300036125</v>
       </c>
       <c r="C121" t="n">
         <v>400</v>
       </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D121" t="n">
+        <v>600012400</v>
       </c>
       <c r="E121" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
         <v>3000037</v>
       </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>2500036985</t>
-        </is>
+      <c r="B122" t="n">
+        <v>2500036985</v>
       </c>
       <c r="C122" t="n">
         <v>400</v>
       </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D122" t="n">
+        <v>600012400</v>
       </c>
       <c r="E122" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
         <v>3003905</v>
       </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>2200006176</t>
-        </is>
+      <c r="B123" t="n">
+        <v>2200006176</v>
       </c>
       <c r="C123" t="n">
         <v>400</v>
       </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D123" t="n">
+        <v>600012400</v>
       </c>
       <c r="E123" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
         <v>3005374</v>
       </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>2600018808</t>
-        </is>
+      <c r="B124" t="n">
+        <v>2600018808</v>
       </c>
       <c r="C124" t="n">
         <v>400</v>
       </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D124" t="n">
+        <v>600012400</v>
       </c>
       <c r="E124" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
         <v>3000514</v>
       </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>2300029770</t>
-        </is>
+      <c r="B125" t="n">
+        <v>2300029770</v>
       </c>
       <c r="C125" t="n">
         <v>400</v>
       </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D125" t="n">
+        <v>600012400</v>
       </c>
       <c r="E125" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
         <v>3000530</v>
       </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>2400027417</t>
-        </is>
+      <c r="B126" t="n">
+        <v>2400027417</v>
       </c>
       <c r="C126" t="n">
         <v>400</v>
       </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D126" t="n">
+        <v>600012400</v>
       </c>
       <c r="E126" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
         <v>3001654</v>
       </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>2500015753</t>
-        </is>
+      <c r="B127" t="n">
+        <v>2500015753</v>
       </c>
       <c r="C127" t="n">
         <v>400</v>
       </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D127" t="n">
+        <v>600012400</v>
       </c>
       <c r="E127" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
         <v>3005183</v>
       </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>2500036212</t>
-        </is>
+      <c r="B128" t="n">
+        <v>2500036212</v>
       </c>
       <c r="C128" t="n">
         <v>400</v>
       </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D128" t="n">
+        <v>600012400</v>
       </c>
       <c r="E128" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
         <v>3000045</v>
       </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>2400022273</t>
-        </is>
+      <c r="B129" t="n">
+        <v>2400022273</v>
       </c>
       <c r="C129" t="n">
         <v>400</v>
       </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D129" t="n">
+        <v>600012400</v>
       </c>
       <c r="E129" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
         <v>3000159</v>
       </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>2600006048</t>
-        </is>
+      <c r="B130" t="n">
+        <v>2600006048</v>
       </c>
       <c r="C130" t="n">
         <v>400</v>
       </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D130" t="n">
+        <v>600012400</v>
       </c>
       <c r="E130" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
         <v>3000552</v>
       </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>2600004772</t>
-        </is>
+      <c r="B131" t="n">
+        <v>2600004772</v>
       </c>
       <c r="C131" t="n">
         <v>400</v>
       </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D131" t="n">
+        <v>600012400</v>
       </c>
       <c r="E131" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
         <v>4001566</v>
       </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>2600007843</t>
-        </is>
+      <c r="B132" t="n">
+        <v>2600007843</v>
       </c>
       <c r="C132" t="n">
         <v>400</v>
       </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D132" t="n">
+        <v>600012400</v>
       </c>
       <c r="E132" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
         <v>3000223</v>
       </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>2400022595</t>
-        </is>
+      <c r="B133" t="n">
+        <v>2400022595</v>
       </c>
       <c r="C133" t="n">
         <v>400</v>
       </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D133" t="n">
+        <v>600012400</v>
       </c>
       <c r="E133" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
         <v>3000401</v>
       </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>2500046008</t>
-        </is>
+      <c r="B134" t="n">
+        <v>2500046008</v>
       </c>
       <c r="C134" t="n">
         <v>400</v>
       </c>
-      <c r="D134" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D134" t="n">
+        <v>600012400</v>
       </c>
       <c r="E134" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
         <v>3000541</v>
       </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>2500021517</t>
-        </is>
+      <c r="B135" t="n">
+        <v>2500021517</v>
       </c>
       <c r="C135" t="n">
         <v>400</v>
       </c>
-      <c r="D135" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D135" t="n">
+        <v>600012400</v>
       </c>
       <c r="E135" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
         <v>3003818</v>
       </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>2300010087</t>
-        </is>
+      <c r="B136" t="n">
+        <v>2300010087</v>
       </c>
       <c r="C136" t="n">
         <v>400</v>
       </c>
-      <c r="D136" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D136" t="n">
+        <v>600012400</v>
       </c>
       <c r="E136" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
         <v>3004347</v>
       </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>2400016921</t>
-        </is>
+      <c r="B137" t="n">
+        <v>2400016921</v>
       </c>
       <c r="C137" t="n">
         <v>400</v>
       </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D137" t="n">
+        <v>600012400</v>
       </c>
       <c r="E137" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
         <v>3000504</v>
       </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>2500039786</t>
-        </is>
+      <c r="B138" t="n">
+        <v>2500039786</v>
       </c>
       <c r="C138" t="n">
         <v>400</v>
       </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D138" t="n">
+        <v>600012400</v>
       </c>
       <c r="E138" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
         <v>3003697</v>
       </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>2500024474</t>
-        </is>
+      <c r="B139" t="n">
+        <v>2500024474</v>
       </c>
       <c r="C139" t="n">
         <v>400</v>
       </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D139" t="n">
+        <v>600012400</v>
       </c>
       <c r="E139" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
         <v>3000248</v>
       </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>2400021064</t>
-        </is>
+      <c r="B140" t="n">
+        <v>2400021064</v>
       </c>
       <c r="C140" t="n">
         <v>400</v>
       </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D140" t="n">
+        <v>600012400</v>
       </c>
       <c r="E140" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
         <v>3000283</v>
       </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>2200021343</t>
-        </is>
+      <c r="B141" t="n">
+        <v>2200021343</v>
       </c>
       <c r="C141" t="n">
         <v>400</v>
       </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D141" t="n">
+        <v>600012400</v>
       </c>
       <c r="E141" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
         <v>3000464</v>
       </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>2600004513</t>
-        </is>
+      <c r="B142" t="n">
+        <v>2600004513</v>
       </c>
       <c r="C142" t="n">
         <v>400</v>
       </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D142" t="n">
+        <v>600012400</v>
       </c>
       <c r="E142" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
         <v>3000286</v>
       </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>2100044072</t>
-        </is>
+      <c r="B143" t="n">
+        <v>2100044072</v>
       </c>
       <c r="C143" t="n">
         <v>400</v>
       </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D143" t="n">
+        <v>600012400</v>
       </c>
       <c r="E143" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
         <v>3000068</v>
       </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>2500007417</t>
-        </is>
+      <c r="B144" t="n">
+        <v>2500007417</v>
       </c>
       <c r="C144" t="n">
         <v>400</v>
       </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D144" t="n">
+        <v>600012400</v>
       </c>
       <c r="E144" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
         <v>3000429</v>
       </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>2500016590</t>
-        </is>
+      <c r="B145" t="n">
+        <v>2500016590</v>
       </c>
       <c r="C145" t="n">
         <v>400</v>
       </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D145" t="n">
+        <v>600012400</v>
       </c>
       <c r="E145" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
         <v>3004763</v>
       </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>2600006599</t>
-        </is>
+      <c r="B146" t="n">
+        <v>2600006599</v>
       </c>
       <c r="C146" t="n">
         <v>400</v>
       </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D146" t="n">
+        <v>600012400</v>
       </c>
       <c r="E146" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
         <v>3000436</v>
       </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>2500021933</t>
-        </is>
+      <c r="B147" t="n">
+        <v>2500021933</v>
       </c>
       <c r="C147" t="n">
         <v>400</v>
       </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D147" t="n">
+        <v>600012400</v>
       </c>
       <c r="E147" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
         <v>3000560</v>
       </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>2600008270</t>
-        </is>
+      <c r="B148" t="n">
+        <v>2600008270</v>
       </c>
       <c r="C148" t="n">
         <v>400</v>
       </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D148" t="n">
+        <v>600012400</v>
       </c>
       <c r="E148" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
         <v>3001656</v>
       </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>2500009811</t>
-        </is>
+      <c r="B149" t="n">
+        <v>2500009811</v>
       </c>
       <c r="C149" t="n">
         <v>400</v>
       </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D149" t="n">
+        <v>600012400</v>
       </c>
       <c r="E149" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
         <v>3005182</v>
       </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>2500036211</t>
-        </is>
+      <c r="B150" t="n">
+        <v>2500036211</v>
       </c>
       <c r="C150" t="n">
         <v>400</v>
       </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D150" t="n">
+        <v>600012400</v>
       </c>
       <c r="E150" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
         <v>3003695</v>
       </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>2500024475</t>
-        </is>
+      <c r="B151" t="n">
+        <v>2500024475</v>
       </c>
       <c r="C151" t="n">
         <v>400</v>
       </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D151" t="n">
+        <v>600012400</v>
       </c>
       <c r="E151" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
         <v>3004469</v>
       </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>2300029145</t>
-        </is>
+      <c r="B152" t="n">
+        <v>2300029145</v>
       </c>
       <c r="C152" t="n">
         <v>400</v>
       </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D152" t="n">
+        <v>600012400</v>
       </c>
       <c r="E152" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
         <v>3000157</v>
       </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>2300009303</t>
-        </is>
+      <c r="B153" t="n">
+        <v>2300009303</v>
       </c>
       <c r="C153" t="n">
         <v>400</v>
       </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D153" t="n">
+        <v>600012400</v>
       </c>
       <c r="E153" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
         <v>3000490</v>
       </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>2500039413</t>
-        </is>
+      <c r="B154" t="n">
+        <v>2500039413</v>
       </c>
       <c r="C154" t="n">
         <v>400</v>
       </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D154" t="n">
+        <v>600012400</v>
       </c>
       <c r="E154" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
         <v>3004367</v>
       </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>2400031808</t>
-        </is>
+      <c r="B155" t="n">
+        <v>2400031808</v>
       </c>
       <c r="C155" t="n">
         <v>400</v>
       </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D155" t="n">
+        <v>600012400</v>
       </c>
       <c r="E155" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
         <v>3000546</v>
       </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>2400014170</t>
-        </is>
+      <c r="B156" t="n">
+        <v>2400014170</v>
       </c>
       <c r="C156" t="n">
         <v>400</v>
       </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D156" t="n">
+        <v>600012400</v>
       </c>
       <c r="E156" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
         <v>3001646</v>
       </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>2500011316</t>
-        </is>
+      <c r="B157" t="n">
+        <v>2500011316</v>
       </c>
       <c r="C157" t="n">
         <v>400</v>
       </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D157" t="n">
+        <v>600012400</v>
       </c>
       <c r="E157" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
         <v>3004911</v>
       </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>2400026379</t>
-        </is>
+      <c r="B158" t="n">
+        <v>2400026379</v>
       </c>
       <c r="C158" t="n">
         <v>400</v>
       </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D158" t="n">
+        <v>600012400</v>
       </c>
       <c r="E158" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
         <v>3000066</v>
       </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>2300039452</t>
-        </is>
+      <c r="B159" t="n">
+        <v>2300039452</v>
       </c>
       <c r="C159" t="n">
         <v>400</v>
       </c>
-      <c r="D159" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D159" t="n">
+        <v>600012400</v>
       </c>
       <c r="E159" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
         <v>3004367</v>
       </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>2400031809</t>
-        </is>
+      <c r="B160" t="n">
+        <v>2400031809</v>
       </c>
       <c r="C160" t="n">
         <v>400</v>
       </c>
-      <c r="D160" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D160" t="n">
+        <v>600012400</v>
       </c>
       <c r="E160" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
         <v>3005198</v>
       </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>2500007037</t>
-        </is>
+      <c r="B161" t="n">
+        <v>2500007037</v>
       </c>
       <c r="C161" t="n">
         <v>400</v>
       </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D161" t="n">
+        <v>600012400</v>
       </c>
       <c r="E161" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
         <v>3000473</v>
       </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>2600007959</t>
-        </is>
+      <c r="B162" t="n">
+        <v>2600007959</v>
       </c>
       <c r="C162" t="n">
         <v>400</v>
       </c>
-      <c r="D162" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D162" t="n">
+        <v>600012400</v>
       </c>
       <c r="E162" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
         <v>3000078</v>
       </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>2600013788</t>
-        </is>
+      <c r="B163" t="n">
+        <v>2600013788</v>
       </c>
       <c r="C163" t="n">
         <v>400</v>
       </c>
-      <c r="D163" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D163" t="n">
+        <v>600012400</v>
       </c>
       <c r="E163" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
         <v>3000226</v>
       </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>2500013395</t>
-        </is>
+      <c r="B164" t="n">
+        <v>2500013395</v>
       </c>
       <c r="C164" t="n">
         <v>400</v>
       </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D164" t="n">
+        <v>600012400</v>
       </c>
       <c r="E164" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
         <v>3000253</v>
       </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>2600009307</t>
-        </is>
+      <c r="B165" t="n">
+        <v>2600009307</v>
       </c>
       <c r="C165" t="n">
         <v>400</v>
       </c>
-      <c r="D165" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D165" t="n">
+        <v>600012400</v>
       </c>
       <c r="E165" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
         <v>3000401</v>
       </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>2600010724</t>
-        </is>
+      <c r="B166" t="n">
+        <v>2600010724</v>
       </c>
       <c r="C166" t="n">
         <v>400</v>
       </c>
-      <c r="D166" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D166" t="n">
+        <v>600012400</v>
       </c>
       <c r="E166" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
         <v>3002742</v>
       </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>2600009136</t>
-        </is>
+      <c r="B167" t="n">
+        <v>2600009136</v>
       </c>
       <c r="C167" t="n">
         <v>400</v>
       </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D167" t="n">
+        <v>600012400</v>
       </c>
       <c r="E167" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
         <v>3001656</v>
       </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>2600008925</t>
-        </is>
+      <c r="B168" t="n">
+        <v>2600008925</v>
       </c>
       <c r="C168" t="n">
         <v>400</v>
       </c>
-      <c r="D168" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D168" t="n">
+        <v>600012400</v>
       </c>
       <c r="E168" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
         <v>3003209</v>
       </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>2600012407</t>
-        </is>
+      <c r="B169" t="n">
+        <v>2600012407</v>
       </c>
       <c r="C169" t="n">
         <v>400</v>
       </c>
-      <c r="D169" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D169" t="n">
+        <v>600012400</v>
       </c>
       <c r="E169" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
         <v>3004304</v>
       </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>2300021855</t>
-        </is>
+      <c r="B170" t="n">
+        <v>2300021855</v>
       </c>
       <c r="C170" t="n">
         <v>400</v>
       </c>
-      <c r="D170" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D170" t="n">
+        <v>600012400</v>
       </c>
       <c r="E170" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
         <v>3000523</v>
       </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>2400022609</t>
-        </is>
+      <c r="B171" t="n">
+        <v>2400022609</v>
       </c>
       <c r="C171" t="n">
         <v>400</v>
       </c>
-      <c r="D171" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D171" t="n">
+        <v>600012400</v>
       </c>
       <c r="E171" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
         <v>3000363</v>
       </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>2500025622</t>
-        </is>
+      <c r="B172" t="n">
+        <v>2500025622</v>
       </c>
       <c r="C172" t="n">
         <v>400</v>
       </c>
-      <c r="D172" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D172" t="n">
+        <v>600012400</v>
       </c>
       <c r="E172" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
         <v>3000473</v>
       </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>2500002724</t>
-        </is>
+      <c r="B173" t="n">
+        <v>2500002724</v>
       </c>
       <c r="C173" t="n">
         <v>400</v>
       </c>
-      <c r="D173" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D173" t="n">
+        <v>600012400</v>
       </c>
       <c r="E173" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
         <v>3000473</v>
       </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>2500013397</t>
-        </is>
+      <c r="B174" t="n">
+        <v>2500013397</v>
       </c>
       <c r="C174" t="n">
         <v>400</v>
       </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D174" t="n">
+        <v>600012400</v>
       </c>
       <c r="E174" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
         <v>3000567</v>
       </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>2600010566</t>
-        </is>
+      <c r="B175" t="n">
+        <v>2600010566</v>
       </c>
       <c r="C175" t="n">
         <v>400</v>
       </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D175" t="n">
+        <v>600012400</v>
       </c>
       <c r="E175" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
         <v>3000068</v>
       </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>2500043544</t>
-        </is>
+      <c r="B176" t="n">
+        <v>2500043544</v>
       </c>
       <c r="C176" t="n">
         <v>400</v>
       </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D176" t="n">
+        <v>600012400</v>
       </c>
       <c r="E176" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
         <v>3000286</v>
       </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>2400038367</t>
-        </is>
+      <c r="B177" t="n">
+        <v>2400038367</v>
       </c>
       <c r="C177" t="n">
         <v>400</v>
       </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D177" t="n">
+        <v>600012400</v>
       </c>
       <c r="E177" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
         <v>3000401</v>
       </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>2500012622</t>
-        </is>
+      <c r="B178" t="n">
+        <v>2500012622</v>
       </c>
       <c r="C178" t="n">
         <v>400</v>
       </c>
-      <c r="D178" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D178" t="n">
+        <v>600012400</v>
       </c>
       <c r="E178" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
         <v>3000514</v>
       </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>2500013650</t>
-        </is>
+      <c r="B179" t="n">
+        <v>2500013650</v>
       </c>
       <c r="C179" t="n">
         <v>400</v>
       </c>
-      <c r="D179" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D179" t="n">
+        <v>600012400</v>
       </c>
       <c r="E179" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
         <v>3003818</v>
       </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>2300022939</t>
-        </is>
+      <c r="B180" t="n">
+        <v>2300022939</v>
       </c>
       <c r="C180" t="n">
         <v>400</v>
       </c>
-      <c r="D180" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D180" t="n">
+        <v>600012400</v>
       </c>
       <c r="E180" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
         <v>3004356</v>
       </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>2300005754</t>
-        </is>
+      <c r="B181" t="n">
+        <v>2300005754</v>
       </c>
       <c r="C181" t="n">
         <v>400</v>
       </c>
-      <c r="D181" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D181" t="n">
+        <v>600012400</v>
       </c>
       <c r="E181" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
         <v>3001649</v>
       </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>2400036656</t>
-        </is>
+      <c r="B182" t="n">
+        <v>2400036656</v>
       </c>
       <c r="C182" t="n">
         <v>400</v>
       </c>
-      <c r="D182" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D182" t="n">
+        <v>600012400</v>
       </c>
       <c r="E182" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
         <v>3002882</v>
       </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>2500012584</t>
-        </is>
+      <c r="B183" t="n">
+        <v>2500012584</v>
       </c>
       <c r="C183" t="n">
         <v>400</v>
       </c>
-      <c r="D183" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D183" t="n">
+        <v>600012400</v>
       </c>
       <c r="E183" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
         <v>3000226</v>
       </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>2400037346</t>
-        </is>
+      <c r="B184" t="n">
+        <v>2400037346</v>
       </c>
       <c r="C184" t="n">
         <v>400</v>
       </c>
-      <c r="D184" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D184" t="n">
+        <v>600012400</v>
       </c>
       <c r="E184" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
         <v>3005396</v>
       </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>2600019201</t>
-        </is>
+      <c r="B185" t="n">
+        <v>2600019201</v>
       </c>
       <c r="C185" t="n">
         <v>400</v>
       </c>
-      <c r="D185" t="inlineStr">
-        <is>
-          <t>600012400</t>
-        </is>
+      <c r="D185" t="n">
+        <v>600012400</v>
       </c>
       <c r="E185" s="1" t="n">
-        <v>46219.72766950409</v>
+        <v>46219.72766950232</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
         <v>3005413</v>
       </c>
-      <c r="B186" t="inlineStr">
+      <c r="B186" t="n">
+        <v>2600019803</v>
+      </c>
+      <c r="C186" t="n">
+        <v>400</v>
+      </c>
+      <c r="D186" t="n">
+        <v>600012400</v>
+      </c>
+      <c r="E186" s="1" t="n">
+        <v>46219.72766950232</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>3000366</v>
+      </c>
+      <c r="B187" t="n">
+        <v>2600018162</v>
+      </c>
+      <c r="C187" t="n">
+        <v>300</v>
+      </c>
+      <c r="D187" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E187" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>3000366</v>
+      </c>
+      <c r="B188" t="n">
+        <v>2600015715</v>
+      </c>
+      <c r="C188" t="n">
+        <v>300</v>
+      </c>
+      <c r="D188" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E188" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B189" t="n">
+        <v>2600012494</v>
+      </c>
+      <c r="C189" t="n">
+        <v>300</v>
+      </c>
+      <c r="D189" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E189" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B190" t="n">
+        <v>2600004986</v>
+      </c>
+      <c r="C190" t="n">
+        <v>300</v>
+      </c>
+      <c r="D190" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E190" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B191" t="n">
+        <v>2600012581</v>
+      </c>
+      <c r="C191" t="n">
+        <v>300</v>
+      </c>
+      <c r="D191" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E191" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B192" t="n">
+        <v>2600004989</v>
+      </c>
+      <c r="C192" t="n">
+        <v>300</v>
+      </c>
+      <c r="D192" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E192" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B193" t="n">
+        <v>2600012492</v>
+      </c>
+      <c r="C193" t="n">
+        <v>300</v>
+      </c>
+      <c r="D193" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E193" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B194" t="n">
+        <v>2600004995</v>
+      </c>
+      <c r="C194" t="n">
+        <v>300</v>
+      </c>
+      <c r="D194" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E194" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>3000093</v>
+      </c>
+      <c r="B195" t="n">
+        <v>2600019667</v>
+      </c>
+      <c r="C195" t="n">
+        <v>300</v>
+      </c>
+      <c r="D195" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E195" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>3000486</v>
+      </c>
+      <c r="B196" t="n">
+        <v>2600020244</v>
+      </c>
+      <c r="C196" t="n">
+        <v>300</v>
+      </c>
+      <c r="D196" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E196" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>3000093</v>
+      </c>
+      <c r="B197" t="n">
+        <v>2600008079</v>
+      </c>
+      <c r="C197" t="n">
+        <v>300</v>
+      </c>
+      <c r="D197" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E197" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>3000537</v>
+      </c>
+      <c r="B198" t="n">
+        <v>2600014583</v>
+      </c>
+      <c r="C198" t="n">
+        <v>300</v>
+      </c>
+      <c r="D198" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E198" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>3000292</v>
+      </c>
+      <c r="B199" t="n">
+        <v>2600012774</v>
+      </c>
+      <c r="C199" t="n">
+        <v>300</v>
+      </c>
+      <c r="D199" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E199" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>3000537</v>
+      </c>
+      <c r="B200" t="n">
+        <v>2600012348</v>
+      </c>
+      <c r="C200" t="n">
+        <v>300</v>
+      </c>
+      <c r="D200" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E200" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>3000733</v>
+      </c>
+      <c r="B201" t="n">
+        <v>2600017894</v>
+      </c>
+      <c r="C201" t="n">
+        <v>300</v>
+      </c>
+      <c r="D201" t="n">
+        <v>600002123</v>
+      </c>
+      <c r="E201" s="1" t="n">
+        <v>46219.77955907407</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>4038837</v>
+      </c>
+      <c r="B202" t="inlineStr">
         <is>
-          <t>2600019803</t>
+          <t>2500043845</t>
         </is>
       </c>
-      <c r="C186" t="n">
-        <v>400</v>
-      </c>
-      <c r="D186" t="inlineStr">
+      <c r="C202" t="n">
+        <v>310</v>
+      </c>
+      <c r="D202" t="inlineStr">
         <is>
-          <t>600012400</t>
+          <t>600031067</t>
         </is>
       </c>
-      <c r="E186" s="1" t="n">
-        <v>46219.72766950409</v>
+      <c r="E202" s="1" t="n">
+        <v>46220.13574616074</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>4000689</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>2600020819</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>310</v>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>600031067</t>
+        </is>
+      </c>
+      <c r="E203" s="1" t="n">
+        <v>46220.13574616074</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>4009121</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>2600009846</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>310</v>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>600031067</t>
+        </is>
+      </c>
+      <c r="E204" s="1" t="n">
+        <v>46220.13574616074</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>4000194</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>2600017631</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>310</v>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>600031067</t>
+        </is>
+      </c>
+      <c r="E205" s="1" t="n">
+        <v>46220.13574616074</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>4000689</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>2600018163</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>310</v>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>600031067</t>
+        </is>
+      </c>
+      <c r="E206" s="1" t="n">
+        <v>46220.13574616074</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>4009121</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>2600016130</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>310</v>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>600031067</t>
+        </is>
+      </c>
+      <c r="E207" s="1" t="n">
+        <v>46220.13574616074</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>4000194</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>2600016030</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>310</v>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>600031067</t>
+        </is>
+      </c>
+      <c r="E208" s="1" t="n">
+        <v>46220.13574616074</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>4000194</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>2600010300</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>310</v>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>600031067</t>
+        </is>
+      </c>
+      <c r="E209" s="1" t="n">
+        <v>46220.13574616074</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>4000688</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>2600020945</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>310</v>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>600031067</t>
+        </is>
+      </c>
+      <c r="E210" s="1" t="n">
+        <v>46220.13574616074</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>4009121</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>2600005939</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>310</v>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>600031067</t>
+        </is>
+      </c>
+      <c r="E211" s="1" t="n">
+        <v>46220.13574616074</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>4000688</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>2600018239</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>310</v>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>600031067</t>
+        </is>
+      </c>
+      <c r="E212" s="1" t="n">
+        <v>46220.13574616074</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>4009062</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>2600013776</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>310</v>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>600031067</t>
+        </is>
+      </c>
+      <c r="E213" s="1" t="n">
+        <v>46220.13574616074</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>4000688</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>2600020621</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>310</v>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>600031067</t>
+        </is>
+      </c>
+      <c r="E214" s="1" t="n">
+        <v>46220.13574616074</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>4000194</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>2600016029</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>310</v>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>600031067</t>
+        </is>
+      </c>
+      <c r="E215" s="1" t="n">
+        <v>46220.13574616074</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>4021439</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>2600017475</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>310</v>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>600031067</t>
+        </is>
+      </c>
+      <c r="E216" s="1" t="n">
+        <v>46220.13574616074</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: refatora interface e implementa importacao de dados SAP
- Separa UI em componentes independentes
- Aplica tema visual corporativo com cards de metricas
- Adiciona switch Modo sem maquina
- Ativa remocao de lotes ja documentados do historico
- Adiciona botao Atualizar Dados para importar LX02 e YMM141
- Remove campo Documento SAP da tela
- Corrige mapeamento de criterios de priorizacao
- Adiciona barra de progresso e carregamento em thread
- Migra layout de pack() para grid()
</commit_message>
<xml_diff>
--- a/data/historico/historico_documentos.xlsx
+++ b/data/historico/historico_documentos.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E216"/>
+  <dimension ref="A1:E398"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3851,315 +3851,3523 @@
       <c r="A202" t="n">
         <v>4038837</v>
       </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>2500043845</t>
-        </is>
+      <c r="B202" t="n">
+        <v>2500043845</v>
       </c>
       <c r="C202" t="n">
         <v>310</v>
       </c>
-      <c r="D202" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D202" t="n">
+        <v>600031067</v>
       </c>
       <c r="E202" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
         <v>4000689</v>
       </c>
-      <c r="B203" t="inlineStr">
-        <is>
-          <t>2600020819</t>
-        </is>
+      <c r="B203" t="n">
+        <v>2600020819</v>
       </c>
       <c r="C203" t="n">
         <v>310</v>
       </c>
-      <c r="D203" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D203" t="n">
+        <v>600031067</v>
       </c>
       <c r="E203" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
         <v>4009121</v>
       </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>2600009846</t>
-        </is>
+      <c r="B204" t="n">
+        <v>2600009846</v>
       </c>
       <c r="C204" t="n">
         <v>310</v>
       </c>
-      <c r="D204" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D204" t="n">
+        <v>600031067</v>
       </c>
       <c r="E204" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
         <v>4000194</v>
       </c>
-      <c r="B205" t="inlineStr">
-        <is>
-          <t>2600017631</t>
-        </is>
+      <c r="B205" t="n">
+        <v>2600017631</v>
       </c>
       <c r="C205" t="n">
         <v>310</v>
       </c>
-      <c r="D205" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D205" t="n">
+        <v>600031067</v>
       </c>
       <c r="E205" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
         <v>4000689</v>
       </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>2600018163</t>
-        </is>
+      <c r="B206" t="n">
+        <v>2600018163</v>
       </c>
       <c r="C206" t="n">
         <v>310</v>
       </c>
-      <c r="D206" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D206" t="n">
+        <v>600031067</v>
       </c>
       <c r="E206" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
         <v>4009121</v>
       </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>2600016130</t>
-        </is>
+      <c r="B207" t="n">
+        <v>2600016130</v>
       </c>
       <c r="C207" t="n">
         <v>310</v>
       </c>
-      <c r="D207" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D207" t="n">
+        <v>600031067</v>
       </c>
       <c r="E207" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
         <v>4000194</v>
       </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>2600016030</t>
-        </is>
+      <c r="B208" t="n">
+        <v>2600016030</v>
       </c>
       <c r="C208" t="n">
         <v>310</v>
       </c>
-      <c r="D208" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D208" t="n">
+        <v>600031067</v>
       </c>
       <c r="E208" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
         <v>4000194</v>
       </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>2600010300</t>
-        </is>
+      <c r="B209" t="n">
+        <v>2600010300</v>
       </c>
       <c r="C209" t="n">
         <v>310</v>
       </c>
-      <c r="D209" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D209" t="n">
+        <v>600031067</v>
       </c>
       <c r="E209" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
         <v>4000688</v>
       </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>2600020945</t>
-        </is>
+      <c r="B210" t="n">
+        <v>2600020945</v>
       </c>
       <c r="C210" t="n">
         <v>310</v>
       </c>
-      <c r="D210" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D210" t="n">
+        <v>600031067</v>
       </c>
       <c r="E210" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
         <v>4009121</v>
       </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>2600005939</t>
-        </is>
+      <c r="B211" t="n">
+        <v>2600005939</v>
       </c>
       <c r="C211" t="n">
         <v>310</v>
       </c>
-      <c r="D211" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D211" t="n">
+        <v>600031067</v>
       </c>
       <c r="E211" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
         <v>4000688</v>
       </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>2600018239</t>
-        </is>
+      <c r="B212" t="n">
+        <v>2600018239</v>
       </c>
       <c r="C212" t="n">
         <v>310</v>
       </c>
-      <c r="D212" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D212" t="n">
+        <v>600031067</v>
       </c>
       <c r="E212" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
         <v>4009062</v>
       </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>2600013776</t>
-        </is>
+      <c r="B213" t="n">
+        <v>2600013776</v>
       </c>
       <c r="C213" t="n">
         <v>310</v>
       </c>
-      <c r="D213" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D213" t="n">
+        <v>600031067</v>
       </c>
       <c r="E213" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
         <v>4000688</v>
       </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>2600020621</t>
-        </is>
+      <c r="B214" t="n">
+        <v>2600020621</v>
       </c>
       <c r="C214" t="n">
         <v>310</v>
       </c>
-      <c r="D214" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D214" t="n">
+        <v>600031067</v>
       </c>
       <c r="E214" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
         <v>4000194</v>
       </c>
-      <c r="B215" t="inlineStr">
-        <is>
-          <t>2600016029</t>
-        </is>
+      <c r="B215" t="n">
+        <v>2600016029</v>
       </c>
       <c r="C215" t="n">
         <v>310</v>
       </c>
-      <c r="D215" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D215" t="n">
+        <v>600031067</v>
       </c>
       <c r="E215" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
         <v>4021439</v>
       </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>2600017475</t>
-        </is>
+      <c r="B216" t="n">
+        <v>2600017475</v>
       </c>
       <c r="C216" t="n">
         <v>310</v>
       </c>
-      <c r="D216" t="inlineStr">
-        <is>
-          <t>600031067</t>
-        </is>
+      <c r="D216" t="n">
+        <v>600031067</v>
       </c>
       <c r="E216" s="1" t="n">
-        <v>46220.13574616074</v>
+        <v>46220.13574615741</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>4022441</v>
+      </c>
+      <c r="B217" t="n">
+        <v>2600016997</v>
+      </c>
+      <c r="C217" t="n">
+        <v>310</v>
+      </c>
+      <c r="D217" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E217" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>4020495</v>
+      </c>
+      <c r="B218" t="n">
+        <v>2600019215</v>
+      </c>
+      <c r="C218" t="n">
+        <v>310</v>
+      </c>
+      <c r="D218" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E218" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>4020495</v>
+      </c>
+      <c r="B219" t="n">
+        <v>2600015553</v>
+      </c>
+      <c r="C219" t="n">
+        <v>310</v>
+      </c>
+      <c r="D219" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E219" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>4018940</v>
+      </c>
+      <c r="B220" t="n">
+        <v>2600004645</v>
+      </c>
+      <c r="C220" t="n">
+        <v>310</v>
+      </c>
+      <c r="D220" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E220" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>4018380</v>
+      </c>
+      <c r="B221" t="n">
+        <v>2500029308</v>
+      </c>
+      <c r="C221" t="n">
+        <v>310</v>
+      </c>
+      <c r="D221" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E221" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>4022190</v>
+      </c>
+      <c r="B222" t="n">
+        <v>2600011519</v>
+      </c>
+      <c r="C222" t="n">
+        <v>310</v>
+      </c>
+      <c r="D222" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E222" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>4018784</v>
+      </c>
+      <c r="B223" t="n">
+        <v>2600017568</v>
+      </c>
+      <c r="C223" t="n">
+        <v>310</v>
+      </c>
+      <c r="D223" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E223" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>4018940</v>
+      </c>
+      <c r="B224" t="n">
+        <v>2600019424</v>
+      </c>
+      <c r="C224" t="n">
+        <v>310</v>
+      </c>
+      <c r="D224" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E224" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>4018388</v>
+      </c>
+      <c r="B225" t="n">
+        <v>2600008281</v>
+      </c>
+      <c r="C225" t="n">
+        <v>310</v>
+      </c>
+      <c r="D225" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E225" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>4015026</v>
+      </c>
+      <c r="B226" t="n">
+        <v>2600018286</v>
+      </c>
+      <c r="C226" t="n">
+        <v>310</v>
+      </c>
+      <c r="D226" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E226" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>4020141</v>
+      </c>
+      <c r="B227" t="n">
+        <v>2600015024</v>
+      </c>
+      <c r="C227" t="n">
+        <v>310</v>
+      </c>
+      <c r="D227" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E227" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>4015026</v>
+      </c>
+      <c r="B228" t="n">
+        <v>2600018287</v>
+      </c>
+      <c r="C228" t="n">
+        <v>310</v>
+      </c>
+      <c r="D228" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E228" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>4022441</v>
+      </c>
+      <c r="B229" t="n">
+        <v>2600010688</v>
+      </c>
+      <c r="C229" t="n">
+        <v>310</v>
+      </c>
+      <c r="D229" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E229" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>4000689</v>
+      </c>
+      <c r="B230" t="n">
+        <v>2600020819</v>
+      </c>
+      <c r="C230" t="n">
+        <v>310</v>
+      </c>
+      <c r="D230" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E230" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>4000689</v>
+      </c>
+      <c r="B231" t="n">
+        <v>2600018163</v>
+      </c>
+      <c r="C231" t="n">
+        <v>310</v>
+      </c>
+      <c r="D231" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E231" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>4000689</v>
+      </c>
+      <c r="B232" t="n">
+        <v>2600020770</v>
+      </c>
+      <c r="C232" t="n">
+        <v>310</v>
+      </c>
+      <c r="D232" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E232" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>4000194</v>
+      </c>
+      <c r="B233" t="n">
+        <v>2600010300</v>
+      </c>
+      <c r="C233" t="n">
+        <v>310</v>
+      </c>
+      <c r="D233" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E233" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>4000231</v>
+      </c>
+      <c r="B234" t="n">
+        <v>2600020446</v>
+      </c>
+      <c r="C234" t="n">
+        <v>310</v>
+      </c>
+      <c r="D234" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E234" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>4006022</v>
+      </c>
+      <c r="B235" t="n">
+        <v>2600020784</v>
+      </c>
+      <c r="C235" t="n">
+        <v>310</v>
+      </c>
+      <c r="D235" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E235" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>4009062</v>
+      </c>
+      <c r="B236" t="n">
+        <v>2600009844</v>
+      </c>
+      <c r="C236" t="n">
+        <v>310</v>
+      </c>
+      <c r="D236" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E236" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>4000688</v>
+      </c>
+      <c r="B237" t="n">
+        <v>2600020945</v>
+      </c>
+      <c r="C237" t="n">
+        <v>310</v>
+      </c>
+      <c r="D237" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E237" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>4013457</v>
+      </c>
+      <c r="B238" t="n">
+        <v>2600013728</v>
+      </c>
+      <c r="C238" t="n">
+        <v>310</v>
+      </c>
+      <c r="D238" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E238" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>4023137</v>
+      </c>
+      <c r="B239" t="n">
+        <v>2600010468</v>
+      </c>
+      <c r="C239" t="n">
+        <v>310</v>
+      </c>
+      <c r="D239" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E239" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>4001552</v>
+      </c>
+      <c r="B240" t="n">
+        <v>2600020439</v>
+      </c>
+      <c r="C240" t="n">
+        <v>310</v>
+      </c>
+      <c r="D240" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E240" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>4001395</v>
+      </c>
+      <c r="B241" t="n">
+        <v>2600016470</v>
+      </c>
+      <c r="C241" t="n">
+        <v>310</v>
+      </c>
+      <c r="D241" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E241" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>4000312</v>
+      </c>
+      <c r="B242" t="n">
+        <v>2600017353</v>
+      </c>
+      <c r="C242" t="n">
+        <v>310</v>
+      </c>
+      <c r="D242" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E242" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>4000688</v>
+      </c>
+      <c r="B243" t="n">
+        <v>2600020621</v>
+      </c>
+      <c r="C243" t="n">
+        <v>310</v>
+      </c>
+      <c r="D243" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E243" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>4001395</v>
+      </c>
+      <c r="B244" t="n">
+        <v>2600012761</v>
+      </c>
+      <c r="C244" t="n">
+        <v>310</v>
+      </c>
+      <c r="D244" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E244" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>4017193</v>
+      </c>
+      <c r="B245" t="n">
+        <v>2600019636</v>
+      </c>
+      <c r="C245" t="n">
+        <v>310</v>
+      </c>
+      <c r="D245" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E245" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>4000310</v>
+      </c>
+      <c r="B246" t="n">
+        <v>2600012968</v>
+      </c>
+      <c r="C246" t="n">
+        <v>310</v>
+      </c>
+      <c r="D246" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E246" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>4009062</v>
+      </c>
+      <c r="B247" t="n">
+        <v>2600020947</v>
+      </c>
+      <c r="C247" t="n">
+        <v>310</v>
+      </c>
+      <c r="D247" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E247" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>4001552</v>
+      </c>
+      <c r="B248" t="n">
+        <v>2600020441</v>
+      </c>
+      <c r="C248" t="n">
+        <v>310</v>
+      </c>
+      <c r="D248" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E248" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>4001395</v>
+      </c>
+      <c r="B249" t="n">
+        <v>2600005145</v>
+      </c>
+      <c r="C249" t="n">
+        <v>310</v>
+      </c>
+      <c r="D249" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E249" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>4021439</v>
+      </c>
+      <c r="B250" t="n">
+        <v>2600020948</v>
+      </c>
+      <c r="C250" t="n">
+        <v>310</v>
+      </c>
+      <c r="D250" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E250" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>4020514</v>
+      </c>
+      <c r="B251" t="n">
+        <v>2600019429</v>
+      </c>
+      <c r="C251" t="n">
+        <v>310</v>
+      </c>
+      <c r="D251" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E251" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>4000194</v>
+      </c>
+      <c r="B252" t="n">
+        <v>2600008215</v>
+      </c>
+      <c r="C252" t="n">
+        <v>310</v>
+      </c>
+      <c r="D252" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E252" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>4021440</v>
+      </c>
+      <c r="B253" t="n">
+        <v>2600020946</v>
+      </c>
+      <c r="C253" t="n">
+        <v>310</v>
+      </c>
+      <c r="D253" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E253" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>4017193</v>
+      </c>
+      <c r="B254" t="n">
+        <v>2600008794</v>
+      </c>
+      <c r="C254" t="n">
+        <v>310</v>
+      </c>
+      <c r="D254" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E254" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>4000312</v>
+      </c>
+      <c r="B255" t="n">
+        <v>2600013428</v>
+      </c>
+      <c r="C255" t="n">
+        <v>310</v>
+      </c>
+      <c r="D255" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E255" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>4000312</v>
+      </c>
+      <c r="B256" t="n">
+        <v>2600013649</v>
+      </c>
+      <c r="C256" t="n">
+        <v>310</v>
+      </c>
+      <c r="D256" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E256" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>4000310</v>
+      </c>
+      <c r="B257" t="n">
+        <v>2600017434</v>
+      </c>
+      <c r="C257" t="n">
+        <v>310</v>
+      </c>
+      <c r="D257" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E257" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>4017193</v>
+      </c>
+      <c r="B258" t="n">
+        <v>2600018765</v>
+      </c>
+      <c r="C258" t="n">
+        <v>310</v>
+      </c>
+      <c r="D258" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E258" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>4001494</v>
+      </c>
+      <c r="B259" t="n">
+        <v>2600018758</v>
+      </c>
+      <c r="C259" t="n">
+        <v>310</v>
+      </c>
+      <c r="D259" t="n">
+        <v>35346</v>
+      </c>
+      <c r="E259" s="1" t="n">
+        <v>46223.63135921297</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>3000366</v>
+      </c>
+      <c r="B260" t="n">
+        <v>2600018162</v>
+      </c>
+      <c r="C260" t="n">
+        <v>300</v>
+      </c>
+      <c r="D260" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E260" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>3000366</v>
+      </c>
+      <c r="B261" t="n">
+        <v>2600015715</v>
+      </c>
+      <c r="C261" t="n">
+        <v>300</v>
+      </c>
+      <c r="D261" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E261" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B262" t="n">
+        <v>2600012494</v>
+      </c>
+      <c r="C262" t="n">
+        <v>300</v>
+      </c>
+      <c r="D262" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E262" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B263" t="n">
+        <v>2600004986</v>
+      </c>
+      <c r="C263" t="n">
+        <v>300</v>
+      </c>
+      <c r="D263" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E263" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B264" t="n">
+        <v>2600012581</v>
+      </c>
+      <c r="C264" t="n">
+        <v>300</v>
+      </c>
+      <c r="D264" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E264" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B265" t="n">
+        <v>2600004989</v>
+      </c>
+      <c r="C265" t="n">
+        <v>300</v>
+      </c>
+      <c r="D265" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E265" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B266" t="n">
+        <v>2600012492</v>
+      </c>
+      <c r="C266" t="n">
+        <v>300</v>
+      </c>
+      <c r="D266" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E266" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B267" t="n">
+        <v>2600004995</v>
+      </c>
+      <c r="C267" t="n">
+        <v>300</v>
+      </c>
+      <c r="D267" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E267" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>3000093</v>
+      </c>
+      <c r="B268" t="n">
+        <v>2600019667</v>
+      </c>
+      <c r="C268" t="n">
+        <v>300</v>
+      </c>
+      <c r="D268" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E268" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>3000486</v>
+      </c>
+      <c r="B269" t="n">
+        <v>2600020244</v>
+      </c>
+      <c r="C269" t="n">
+        <v>300</v>
+      </c>
+      <c r="D269" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E269" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>3000093</v>
+      </c>
+      <c r="B270" t="n">
+        <v>2600008079</v>
+      </c>
+      <c r="C270" t="n">
+        <v>300</v>
+      </c>
+      <c r="D270" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E270" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>3000537</v>
+      </c>
+      <c r="B271" t="n">
+        <v>2600014583</v>
+      </c>
+      <c r="C271" t="n">
+        <v>300</v>
+      </c>
+      <c r="D271" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E271" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>3000292</v>
+      </c>
+      <c r="B272" t="n">
+        <v>2600012774</v>
+      </c>
+      <c r="C272" t="n">
+        <v>300</v>
+      </c>
+      <c r="D272" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E272" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>3000537</v>
+      </c>
+      <c r="B273" t="n">
+        <v>2600012348</v>
+      </c>
+      <c r="C273" t="n">
+        <v>300</v>
+      </c>
+      <c r="D273" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E273" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>3000733</v>
+      </c>
+      <c r="B274" t="n">
+        <v>2600017894</v>
+      </c>
+      <c r="C274" t="n">
+        <v>300</v>
+      </c>
+      <c r="D274" t="n">
+        <v>6342324</v>
+      </c>
+      <c r="E274" s="1" t="n">
+        <v>46224.58327586806</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>4038837</v>
+      </c>
+      <c r="B275" t="n">
+        <v>2500043845</v>
+      </c>
+      <c r="C275" t="n">
+        <v>310</v>
+      </c>
+      <c r="D275" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E275" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>4000689</v>
+      </c>
+      <c r="B276" t="n">
+        <v>2600020819</v>
+      </c>
+      <c r="C276" t="n">
+        <v>310</v>
+      </c>
+      <c r="D276" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E276" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>4009121</v>
+      </c>
+      <c r="B277" t="n">
+        <v>2600009846</v>
+      </c>
+      <c r="C277" t="n">
+        <v>310</v>
+      </c>
+      <c r="D277" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E277" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>4000194</v>
+      </c>
+      <c r="B278" t="n">
+        <v>2600017631</v>
+      </c>
+      <c r="C278" t="n">
+        <v>310</v>
+      </c>
+      <c r="D278" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E278" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>4000689</v>
+      </c>
+      <c r="B279" t="n">
+        <v>2600018163</v>
+      </c>
+      <c r="C279" t="n">
+        <v>310</v>
+      </c>
+      <c r="D279" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E279" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>4009121</v>
+      </c>
+      <c r="B280" t="n">
+        <v>2600016130</v>
+      </c>
+      <c r="C280" t="n">
+        <v>310</v>
+      </c>
+      <c r="D280" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E280" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>4000194</v>
+      </c>
+      <c r="B281" t="n">
+        <v>2600016030</v>
+      </c>
+      <c r="C281" t="n">
+        <v>310</v>
+      </c>
+      <c r="D281" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E281" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>4000194</v>
+      </c>
+      <c r="B282" t="n">
+        <v>2600010300</v>
+      </c>
+      <c r="C282" t="n">
+        <v>310</v>
+      </c>
+      <c r="D282" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E282" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>4000688</v>
+      </c>
+      <c r="B283" t="n">
+        <v>2600020945</v>
+      </c>
+      <c r="C283" t="n">
+        <v>310</v>
+      </c>
+      <c r="D283" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E283" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>4009121</v>
+      </c>
+      <c r="B284" t="n">
+        <v>2600005939</v>
+      </c>
+      <c r="C284" t="n">
+        <v>310</v>
+      </c>
+      <c r="D284" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E284" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>4000688</v>
+      </c>
+      <c r="B285" t="n">
+        <v>2600018239</v>
+      </c>
+      <c r="C285" t="n">
+        <v>310</v>
+      </c>
+      <c r="D285" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E285" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>4009062</v>
+      </c>
+      <c r="B286" t="n">
+        <v>2600013776</v>
+      </c>
+      <c r="C286" t="n">
+        <v>310</v>
+      </c>
+      <c r="D286" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E286" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>4000688</v>
+      </c>
+      <c r="B287" t="n">
+        <v>2600020621</v>
+      </c>
+      <c r="C287" t="n">
+        <v>310</v>
+      </c>
+      <c r="D287" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E287" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>4000194</v>
+      </c>
+      <c r="B288" t="n">
+        <v>2600016029</v>
+      </c>
+      <c r="C288" t="n">
+        <v>310</v>
+      </c>
+      <c r="D288" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E288" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>4021439</v>
+      </c>
+      <c r="B289" t="n">
+        <v>2600017475</v>
+      </c>
+      <c r="C289" t="n">
+        <v>310</v>
+      </c>
+      <c r="D289" t="n">
+        <v>612345688</v>
+      </c>
+      <c r="E289" s="1" t="n">
+        <v>46224.66405245371</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>3000021</v>
+      </c>
+      <c r="B290" t="n">
+        <v>2600008300</v>
+      </c>
+      <c r="C290" t="n">
+        <v>300</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E290" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>2004583</v>
+      </c>
+      <c r="B291" t="n">
+        <v>2624906</v>
+      </c>
+      <c r="C291" t="n">
+        <v>300</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E291" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>2000182</v>
+      </c>
+      <c r="B292" t="n">
+        <v>2624910</v>
+      </c>
+      <c r="C292" t="n">
+        <v>300</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E292" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>2003659</v>
+      </c>
+      <c r="B293" t="n">
+        <v>2625968</v>
+      </c>
+      <c r="C293" t="n">
+        <v>300</v>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E293" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>2000081</v>
+      </c>
+      <c r="B294" t="n">
+        <v>2617402</v>
+      </c>
+      <c r="C294" t="n">
+        <v>300</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E294" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>2000081</v>
+      </c>
+      <c r="B295" t="n">
+        <v>2617406</v>
+      </c>
+      <c r="C295" t="n">
+        <v>300</v>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E295" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>2000162</v>
+      </c>
+      <c r="B296" t="n">
+        <v>2625505</v>
+      </c>
+      <c r="C296" t="n">
+        <v>300</v>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E296" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>2004217</v>
+      </c>
+      <c r="B297" t="n">
+        <v>2622168</v>
+      </c>
+      <c r="C297" t="n">
+        <v>300</v>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E297" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>2003758</v>
+      </c>
+      <c r="B298" t="n">
+        <v>2618560</v>
+      </c>
+      <c r="C298" t="n">
+        <v>300</v>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E298" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>3000043</v>
+      </c>
+      <c r="B299" t="n">
+        <v>2600017675</v>
+      </c>
+      <c r="C299" t="n">
+        <v>300</v>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E299" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>3000043</v>
+      </c>
+      <c r="B300" t="n">
+        <v>2600011703</v>
+      </c>
+      <c r="C300" t="n">
+        <v>300</v>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E300" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="n">
+        <v>3000040</v>
+      </c>
+      <c r="B301" t="n">
+        <v>2600012503</v>
+      </c>
+      <c r="C301" t="n">
+        <v>300</v>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E301" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="n">
+        <v>3000024</v>
+      </c>
+      <c r="B302" t="n">
+        <v>2600017561</v>
+      </c>
+      <c r="C302" t="n">
+        <v>300</v>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E302" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="n">
+        <v>3000024</v>
+      </c>
+      <c r="B303" t="n">
+        <v>2600017563</v>
+      </c>
+      <c r="C303" t="n">
+        <v>300</v>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E303" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="n">
+        <v>3000078</v>
+      </c>
+      <c r="B304" t="n">
+        <v>2600017539</v>
+      </c>
+      <c r="C304" t="n">
+        <v>300</v>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E304" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="n">
+        <v>3000068</v>
+      </c>
+      <c r="B305" t="n">
+        <v>2600020662</v>
+      </c>
+      <c r="C305" t="n">
+        <v>300</v>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E305" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="n">
+        <v>3000093</v>
+      </c>
+      <c r="B306" t="n">
+        <v>2600019667</v>
+      </c>
+      <c r="C306" t="n">
+        <v>300</v>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E306" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="n">
+        <v>3000040</v>
+      </c>
+      <c r="B307" t="n">
+        <v>2600009308</v>
+      </c>
+      <c r="C307" t="n">
+        <v>300</v>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E307" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="n">
+        <v>3000027</v>
+      </c>
+      <c r="B308" t="n">
+        <v>2600017523</v>
+      </c>
+      <c r="C308" t="n">
+        <v>300</v>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E308" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="n">
+        <v>3000043</v>
+      </c>
+      <c r="B309" t="n">
+        <v>2600017674</v>
+      </c>
+      <c r="C309" t="n">
+        <v>300</v>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E309" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="n">
+        <v>3000037</v>
+      </c>
+      <c r="B310" t="n">
+        <v>2600016291</v>
+      </c>
+      <c r="C310" t="n">
+        <v>300</v>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E310" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="n">
+        <v>3000027</v>
+      </c>
+      <c r="B311" t="n">
+        <v>2600020426</v>
+      </c>
+      <c r="C311" t="n">
+        <v>300</v>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E311" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>3000093</v>
+      </c>
+      <c r="B312" t="n">
+        <v>2600008079</v>
+      </c>
+      <c r="C312" t="n">
+        <v>300</v>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E312" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>3000066</v>
+      </c>
+      <c r="B313" t="n">
+        <v>2600012787</v>
+      </c>
+      <c r="C313" t="n">
+        <v>300</v>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E313" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="n">
+        <v>3000037</v>
+      </c>
+      <c r="B314" t="n">
+        <v>2600019509</v>
+      </c>
+      <c r="C314" t="n">
+        <v>300</v>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E314" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>3000129</v>
+      </c>
+      <c r="B315" t="n">
+        <v>2600018626</v>
+      </c>
+      <c r="C315" t="n">
+        <v>300</v>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E315" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="n">
+        <v>2003758</v>
+      </c>
+      <c r="B316" t="n">
+        <v>2624076</v>
+      </c>
+      <c r="C316" t="n">
+        <v>300</v>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E316" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="n">
+        <v>2003717</v>
+      </c>
+      <c r="B317" t="n">
+        <v>2623720</v>
+      </c>
+      <c r="C317" t="n">
+        <v>300</v>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E317" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="n">
+        <v>3000055</v>
+      </c>
+      <c r="B318" t="n">
+        <v>2600019511</v>
+      </c>
+      <c r="C318" t="n">
+        <v>300</v>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E318" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="n">
+        <v>3000060</v>
+      </c>
+      <c r="B319" t="n">
+        <v>2600019119</v>
+      </c>
+      <c r="C319" t="n">
+        <v>300</v>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E319" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="n">
+        <v>3000055</v>
+      </c>
+      <c r="B320" t="n">
+        <v>2600019456</v>
+      </c>
+      <c r="C320" t="n">
+        <v>300</v>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E320" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="n">
+        <v>3000055</v>
+      </c>
+      <c r="B321" t="n">
+        <v>2600013124</v>
+      </c>
+      <c r="C321" t="n">
+        <v>300</v>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E321" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="n">
+        <v>3000055</v>
+      </c>
+      <c r="B322" t="n">
+        <v>2600013125</v>
+      </c>
+      <c r="C322" t="n">
+        <v>300</v>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E322" s="1" t="n">
+        <v>46224.68011892361</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="n">
+        <v>3000366</v>
+      </c>
+      <c r="B323" t="n">
+        <v>2600018162</v>
+      </c>
+      <c r="C323" t="n">
+        <v>300</v>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E323" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="n">
+        <v>3000366</v>
+      </c>
+      <c r="B324" t="n">
+        <v>2600015715</v>
+      </c>
+      <c r="C324" t="n">
+        <v>300</v>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E324" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B325" t="n">
+        <v>2600012494</v>
+      </c>
+      <c r="C325" t="n">
+        <v>300</v>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E325" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B326" t="n">
+        <v>2600004986</v>
+      </c>
+      <c r="C326" t="n">
+        <v>300</v>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E326" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B327" t="n">
+        <v>2600012581</v>
+      </c>
+      <c r="C327" t="n">
+        <v>300</v>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E327" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B328" t="n">
+        <v>2600004989</v>
+      </c>
+      <c r="C328" t="n">
+        <v>300</v>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E328" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B329" t="n">
+        <v>2600012492</v>
+      </c>
+      <c r="C329" t="n">
+        <v>300</v>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E329" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B330" t="n">
+        <v>2600004995</v>
+      </c>
+      <c r="C330" t="n">
+        <v>300</v>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E330" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="n">
+        <v>3000093</v>
+      </c>
+      <c r="B331" t="n">
+        <v>2600019667</v>
+      </c>
+      <c r="C331" t="n">
+        <v>300</v>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E331" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="n">
+        <v>3000486</v>
+      </c>
+      <c r="B332" t="n">
+        <v>2600020244</v>
+      </c>
+      <c r="C332" t="n">
+        <v>300</v>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E332" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="n">
+        <v>3000093</v>
+      </c>
+      <c r="B333" t="n">
+        <v>2600008079</v>
+      </c>
+      <c r="C333" t="n">
+        <v>300</v>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E333" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="n">
+        <v>3000537</v>
+      </c>
+      <c r="B334" t="n">
+        <v>2600014583</v>
+      </c>
+      <c r="C334" t="n">
+        <v>300</v>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E334" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="n">
+        <v>3000292</v>
+      </c>
+      <c r="B335" t="n">
+        <v>2600012774</v>
+      </c>
+      <c r="C335" t="n">
+        <v>300</v>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E335" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="n">
+        <v>3000537</v>
+      </c>
+      <c r="B336" t="n">
+        <v>2600012348</v>
+      </c>
+      <c r="C336" t="n">
+        <v>300</v>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E336" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="n">
+        <v>3000733</v>
+      </c>
+      <c r="B337" t="n">
+        <v>2600017894</v>
+      </c>
+      <c r="C337" t="n">
+        <v>300</v>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="E337" s="1" t="n">
+        <v>46224.68076042824</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="n">
+        <v>3000366</v>
+      </c>
+      <c r="B338" t="n">
+        <v>2600018162</v>
+      </c>
+      <c r="C338" t="n">
+        <v>300</v>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E338" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="n">
+        <v>3000366</v>
+      </c>
+      <c r="B339" t="n">
+        <v>2600015715</v>
+      </c>
+      <c r="C339" t="n">
+        <v>300</v>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E339" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B340" t="n">
+        <v>2600012494</v>
+      </c>
+      <c r="C340" t="n">
+        <v>300</v>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E340" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B341" t="n">
+        <v>2600004986</v>
+      </c>
+      <c r="C341" t="n">
+        <v>300</v>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E341" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B342" t="n">
+        <v>2600012581</v>
+      </c>
+      <c r="C342" t="n">
+        <v>300</v>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E342" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B343" t="n">
+        <v>2600004989</v>
+      </c>
+      <c r="C343" t="n">
+        <v>300</v>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E343" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B344" t="n">
+        <v>2600012492</v>
+      </c>
+      <c r="C344" t="n">
+        <v>300</v>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E344" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B345" t="n">
+        <v>2600004995</v>
+      </c>
+      <c r="C345" t="n">
+        <v>300</v>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E345" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="n">
+        <v>3000093</v>
+      </c>
+      <c r="B346" t="n">
+        <v>2600019667</v>
+      </c>
+      <c r="C346" t="n">
+        <v>300</v>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E346" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="n">
+        <v>3000486</v>
+      </c>
+      <c r="B347" t="n">
+        <v>2600020244</v>
+      </c>
+      <c r="C347" t="n">
+        <v>300</v>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E347" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="n">
+        <v>3000093</v>
+      </c>
+      <c r="B348" t="n">
+        <v>2600008079</v>
+      </c>
+      <c r="C348" t="n">
+        <v>300</v>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E348" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="n">
+        <v>3000537</v>
+      </c>
+      <c r="B349" t="n">
+        <v>2600014583</v>
+      </c>
+      <c r="C349" t="n">
+        <v>300</v>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E349" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="n">
+        <v>3000292</v>
+      </c>
+      <c r="B350" t="n">
+        <v>2600012774</v>
+      </c>
+      <c r="C350" t="n">
+        <v>300</v>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E350" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="n">
+        <v>3000537</v>
+      </c>
+      <c r="B351" t="n">
+        <v>2600012348</v>
+      </c>
+      <c r="C351" t="n">
+        <v>300</v>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E351" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="n">
+        <v>3000733</v>
+      </c>
+      <c r="B352" t="n">
+        <v>2600017894</v>
+      </c>
+      <c r="C352" t="n">
+        <v>300</v>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="E352" s="1" t="n">
+        <v>46224.68109415509</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="n">
+        <v>4018101</v>
+      </c>
+      <c r="B353" t="n">
+        <v>2600020068</v>
+      </c>
+      <c r="C353" t="n">
+        <v>310</v>
+      </c>
+      <c r="D353" t="inlineStr"/>
+      <c r="E353" s="1" t="n">
+        <v>46224.72446489584</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="n">
+        <v>4013827</v>
+      </c>
+      <c r="B354" t="n">
+        <v>2600018149</v>
+      </c>
+      <c r="C354" t="n">
+        <v>310</v>
+      </c>
+      <c r="D354" t="inlineStr"/>
+      <c r="E354" s="1" t="n">
+        <v>46224.72446489584</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="n">
+        <v>4012180</v>
+      </c>
+      <c r="B355" t="n">
+        <v>2600016304</v>
+      </c>
+      <c r="C355" t="n">
+        <v>310</v>
+      </c>
+      <c r="D355" t="inlineStr"/>
+      <c r="E355" s="1" t="n">
+        <v>46224.72446489584</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="n">
+        <v>4035564</v>
+      </c>
+      <c r="B356" t="n">
+        <v>2400041446</v>
+      </c>
+      <c r="C356" t="n">
+        <v>310</v>
+      </c>
+      <c r="D356" t="inlineStr"/>
+      <c r="E356" s="1" t="n">
+        <v>46224.72446489584</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="n">
+        <v>4021094</v>
+      </c>
+      <c r="B357" t="n">
+        <v>2600010101</v>
+      </c>
+      <c r="C357" t="n">
+        <v>310</v>
+      </c>
+      <c r="D357" t="inlineStr"/>
+      <c r="E357" s="1" t="n">
+        <v>46224.72446489584</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="n">
+        <v>4021094</v>
+      </c>
+      <c r="B358" t="n">
+        <v>2600020024</v>
+      </c>
+      <c r="C358" t="n">
+        <v>310</v>
+      </c>
+      <c r="D358" t="inlineStr"/>
+      <c r="E358" s="1" t="n">
+        <v>46224.72446489584</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="n">
+        <v>3000204</v>
+      </c>
+      <c r="B359" t="n">
+        <v>2600013272</v>
+      </c>
+      <c r="C359" t="n">
+        <v>300</v>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E359" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="n">
+        <v>3000204</v>
+      </c>
+      <c r="B360" t="n">
+        <v>2600017554</v>
+      </c>
+      <c r="C360" t="n">
+        <v>300</v>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E360" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="n">
+        <v>3000204</v>
+      </c>
+      <c r="B361" t="n">
+        <v>2600017507</v>
+      </c>
+      <c r="C361" t="n">
+        <v>300</v>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E361" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="n">
+        <v>3000204</v>
+      </c>
+      <c r="B362" t="n">
+        <v>2600017552</v>
+      </c>
+      <c r="C362" t="n">
+        <v>300</v>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E362" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="n">
+        <v>3000204</v>
+      </c>
+      <c r="B363" t="n">
+        <v>2600017553</v>
+      </c>
+      <c r="C363" t="n">
+        <v>300</v>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E363" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="n">
+        <v>3000203</v>
+      </c>
+      <c r="B364" t="n">
+        <v>2600016051</v>
+      </c>
+      <c r="C364" t="n">
+        <v>300</v>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E364" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="n">
+        <v>3000191</v>
+      </c>
+      <c r="B365" t="n">
+        <v>2600019386</v>
+      </c>
+      <c r="C365" t="n">
+        <v>300</v>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E365" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="n">
+        <v>3000204</v>
+      </c>
+      <c r="B366" t="n">
+        <v>2600018147</v>
+      </c>
+      <c r="C366" t="n">
+        <v>300</v>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E366" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="n">
+        <v>3000205</v>
+      </c>
+      <c r="B367" t="n">
+        <v>2600017875</v>
+      </c>
+      <c r="C367" t="n">
+        <v>300</v>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E367" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="n">
+        <v>3000191</v>
+      </c>
+      <c r="B368" t="n">
+        <v>2600019385</v>
+      </c>
+      <c r="C368" t="n">
+        <v>300</v>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E368" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="n">
+        <v>3000191</v>
+      </c>
+      <c r="B369" t="n">
+        <v>2600008743</v>
+      </c>
+      <c r="C369" t="n">
+        <v>300</v>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E369" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="n">
+        <v>3000204</v>
+      </c>
+      <c r="B370" t="n">
+        <v>2600013273</v>
+      </c>
+      <c r="C370" t="n">
+        <v>300</v>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E370" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="n">
+        <v>3000191</v>
+      </c>
+      <c r="B371" t="n">
+        <v>2600019384</v>
+      </c>
+      <c r="C371" t="n">
+        <v>300</v>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E371" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="n">
+        <v>3000204</v>
+      </c>
+      <c r="B372" t="n">
+        <v>2600013266</v>
+      </c>
+      <c r="C372" t="n">
+        <v>300</v>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E372" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="n">
+        <v>3000127</v>
+      </c>
+      <c r="B373" t="n">
+        <v>2600016288</v>
+      </c>
+      <c r="C373" t="n">
+        <v>300</v>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E373" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="n">
+        <v>3000161</v>
+      </c>
+      <c r="B374" t="n">
+        <v>2600010682</v>
+      </c>
+      <c r="C374" t="n">
+        <v>300</v>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E374" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="n">
+        <v>3000133</v>
+      </c>
+      <c r="B375" t="n">
+        <v>2600019672</v>
+      </c>
+      <c r="C375" t="n">
+        <v>300</v>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E375" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="n">
+        <v>3000249</v>
+      </c>
+      <c r="B376" t="n">
+        <v>2600018153</v>
+      </c>
+      <c r="C376" t="n">
+        <v>300</v>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E376" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="n">
+        <v>3000249</v>
+      </c>
+      <c r="B377" t="n">
+        <v>2600018151</v>
+      </c>
+      <c r="C377" t="n">
+        <v>300</v>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E377" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="n">
+        <v>3000133</v>
+      </c>
+      <c r="B378" t="n">
+        <v>2600019670</v>
+      </c>
+      <c r="C378" t="n">
+        <v>300</v>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E378" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="n">
+        <v>3000134</v>
+      </c>
+      <c r="B379" t="n">
+        <v>2600020924</v>
+      </c>
+      <c r="C379" t="n">
+        <v>300</v>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E379" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="n">
+        <v>3000086</v>
+      </c>
+      <c r="B380" t="n">
+        <v>2600020069</v>
+      </c>
+      <c r="C380" t="n">
+        <v>300</v>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E380" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="n">
+        <v>3000086</v>
+      </c>
+      <c r="B381" t="n">
+        <v>2600020070</v>
+      </c>
+      <c r="C381" t="n">
+        <v>300</v>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>1232454</t>
+        </is>
+      </c>
+      <c r="E381" s="1" t="n">
+        <v>46224.73883230324</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="n">
+        <v>4018101</v>
+      </c>
+      <c r="B382" t="n">
+        <v>2600017871</v>
+      </c>
+      <c r="C382" t="n">
+        <v>310</v>
+      </c>
+      <c r="D382" t="inlineStr"/>
+      <c r="E382" s="1" t="n">
+        <v>46224.75992053241</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="n">
+        <v>4034441</v>
+      </c>
+      <c r="B383" t="n">
+        <v>2400021304</v>
+      </c>
+      <c r="C383" t="n">
+        <v>310</v>
+      </c>
+      <c r="D383" t="inlineStr"/>
+      <c r="E383" s="1" t="n">
+        <v>46224.75992053241</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="n">
+        <v>4034457</v>
+      </c>
+      <c r="B384" t="n">
+        <v>2600016364</v>
+      </c>
+      <c r="C384" t="n">
+        <v>310</v>
+      </c>
+      <c r="D384" t="inlineStr"/>
+      <c r="E384" s="1" t="n">
+        <v>46224.75992053241</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="n">
+        <v>4038837</v>
+      </c>
+      <c r="B385" t="n">
+        <v>2600008160</v>
+      </c>
+      <c r="C385" t="n">
+        <v>310</v>
+      </c>
+      <c r="D385" t="inlineStr"/>
+      <c r="E385" s="1" t="n">
+        <v>46224.75992053241</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="n">
+        <v>4027483</v>
+      </c>
+      <c r="B386" t="n">
+        <v>2600015651</v>
+      </c>
+      <c r="C386" t="n">
+        <v>310</v>
+      </c>
+      <c r="D386" t="inlineStr"/>
+      <c r="E386" s="1" t="n">
+        <v>46224.75992053241</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="n">
+        <v>4001389</v>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>2600020445</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr"/>
+      <c r="E387" s="1" t="n">
+        <v>46224.7605434451</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="n">
+        <v>4000231</v>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>2600020447</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr"/>
+      <c r="E388" s="1" t="n">
+        <v>46224.7605434451</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="n">
+        <v>4000399</v>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>2600017356</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr"/>
+      <c r="E389" s="1" t="n">
+        <v>46224.7605434451</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="n">
+        <v>4000203</v>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>2600017367</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr"/>
+      <c r="E390" s="1" t="n">
+        <v>46224.7605434451</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="n">
+        <v>4000228</v>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>2600020443</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr"/>
+      <c r="E391" s="1" t="n">
+        <v>46224.7605434451</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="n">
+        <v>4000399</v>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>2600010472</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr"/>
+      <c r="E392" s="1" t="n">
+        <v>46224.7605434451</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="n">
+        <v>4001389</v>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>2600019548</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr"/>
+      <c r="E393" s="1" t="n">
+        <v>46224.7605434451</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="n">
+        <v>4000231</v>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>2600020435</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr"/>
+      <c r="E394" s="1" t="n">
+        <v>46224.7605434451</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="n">
+        <v>4000203</v>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>2600012969</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr"/>
+      <c r="E395" s="1" t="n">
+        <v>46224.7605434451</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="n">
+        <v>4001247</v>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>2400040579</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr"/>
+      <c r="E396" s="1" t="n">
+        <v>46224.7605434451</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="n">
+        <v>4001395</v>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>2600016471</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr"/>
+      <c r="E397" s="1" t="n">
+        <v>46224.7605434451</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="n">
+        <v>4000310</v>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>2600020442</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr"/>
+      <c r="E398" s="1" t="n">
+        <v>46224.7605434451</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refatora exportação do Excel: filtra colunas relevantes e melhora formatação Mantém apenas Material, Descrição, Lote, Posição, Tipo Depósito e Qtd. Estoque. Aplica cabeçalho com fundo azul e dados alinhados à esquerda.
</commit_message>
<xml_diff>
--- a/data/historico/historico_documentos.xlsx
+++ b/data/historico/historico_documentos.xlsx
@@ -16,10 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -49,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,226 +476,6 @@
         <is>
           <t>total_valor_geracao</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>3001628</v>
-      </c>
-      <c r="B2" t="n">
-        <v>2600014414</v>
-      </c>
-      <c r="C2" t="n">
-        <v>300</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>600005467</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>46229.76556306713</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>c9489548-026e-4449-9410-60c5cda92bac</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>valor</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I2" t="n">
-        <v>74560</v>
-      </c>
-      <c r="J2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K2" t="n">
-        <v>100</v>
-      </c>
-      <c r="L2" t="n">
-        <v>1653323.6127568</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>3000550</v>
-      </c>
-      <c r="B3" t="n">
-        <v>2600016047</v>
-      </c>
-      <c r="C3" t="n">
-        <v>300</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>600005467</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="n">
-        <v>46229.76556306713</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>c9489548-026e-4449-9410-60c5cda92bac</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>valor</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>18</v>
-      </c>
-      <c r="I3" t="n">
-        <v>292732.57</v>
-      </c>
-      <c r="J3" t="n">
-        <v>5</v>
-      </c>
-      <c r="K3" t="n">
-        <v>100</v>
-      </c>
-      <c r="L3" t="n">
-        <v>1653323.6127568</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3000366</v>
-      </c>
-      <c r="B4" t="n">
-        <v>2600015715</v>
-      </c>
-      <c r="C4" t="n">
-        <v>300</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>600005467</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>46229.76556306713</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>c9489548-026e-4449-9410-60c5cda92bac</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>valor</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>25</v>
-      </c>
-      <c r="I4" t="n">
-        <v>308387.0391568</v>
-      </c>
-      <c r="J4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K4" t="n">
-        <v>100</v>
-      </c>
-      <c r="L4" t="n">
-        <v>1653323.6127568</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>3002233</v>
-      </c>
-      <c r="B5" t="n">
-        <v>2600014698</v>
-      </c>
-      <c r="C5" t="n">
-        <v>300</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>600005467</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>46229.76556306713</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>c9489548-026e-4449-9410-60c5cda92bac</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>valor</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>12</v>
-      </c>
-      <c r="I5" t="n">
-        <v>257752</v>
-      </c>
-      <c r="J5" t="n">
-        <v>5</v>
-      </c>
-      <c r="K5" t="n">
-        <v>100</v>
-      </c>
-      <c r="L5" t="n">
-        <v>1653323.6127568</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>3002233</v>
-      </c>
-      <c r="B6" t="n">
-        <v>2600011176</v>
-      </c>
-      <c r="C6" t="n">
-        <v>300</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>600005467</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>46229.76556306713</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>c9489548-026e-4449-9410-60c5cda92bac</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>valor</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>42</v>
-      </c>
-      <c r="I6" t="n">
-        <v>719892.0035999999</v>
-      </c>
-      <c r="J6" t="n">
-        <v>5</v>
-      </c>
-      <c r="K6" t="n">
-        <v>100</v>
-      </c>
-      <c r="L6" t="n">
-        <v>1653323.6127568</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adiciona interface web Flask e pacotes __init__.py no projeto
- Cria aplicação web em web/ com Flask (upload, filtros, histórico, visão geral)
- Adiciona __init__.py em todos os pacotes src/ para padronização
- Cria diretório src/modelos/ para modelos futuros
- Adiciona flag aplicacao_realizada no controller
- Adiciona flask às dependências
</commit_message>
<xml_diff>
--- a/data/historico/historico_documentos.xlsx
+++ b/data/historico/historico_documentos.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,6 +480,226 @@
         <is>
           <t>total_valor_geracao</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>3001628</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2600014414</v>
+      </c>
+      <c r="C2" t="n">
+        <v>300</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>345346</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>46229.92942528935</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2436b635-d34f-4e71-9116-1291819daa38</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I2" t="n">
+        <v>74560</v>
+      </c>
+      <c r="J2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K2" t="n">
+        <v>100</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1653323.6127568</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>3000550</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2600016047</v>
+      </c>
+      <c r="C3" t="n">
+        <v>300</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>345346</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>46229.92942528935</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2436b635-d34f-4e71-9116-1291819daa38</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>18</v>
+      </c>
+      <c r="I3" t="n">
+        <v>292732.57</v>
+      </c>
+      <c r="J3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K3" t="n">
+        <v>100</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1653323.6127568</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3000366</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2600015715</v>
+      </c>
+      <c r="C4" t="n">
+        <v>300</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>345346</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>46229.92942528935</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2436b635-d34f-4e71-9116-1291819daa38</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>25</v>
+      </c>
+      <c r="I4" t="n">
+        <v>308387.0391568</v>
+      </c>
+      <c r="J4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K4" t="n">
+        <v>100</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1653323.6127568</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3002233</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2600014698</v>
+      </c>
+      <c r="C5" t="n">
+        <v>300</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>345346</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>46229.92942528935</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2436b635-d34f-4e71-9116-1291819daa38</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>12</v>
+      </c>
+      <c r="I5" t="n">
+        <v>257752</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" t="n">
+        <v>100</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1653323.6127568</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3002233</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2600011176</v>
+      </c>
+      <c r="C6" t="n">
+        <v>300</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>345346</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>46229.92942528935</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2436b635-d34f-4e71-9116-1291819daa38</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>42</v>
+      </c>
+      <c r="I6" t="n">
+        <v>719892.0035999999</v>
+      </c>
+      <c r="J6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" t="n">
+        <v>100</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1653323.6127568</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: prepara deploy Heroku, adiciona página de resumo e melhorias na UI
- Adiciona Procfile e runtime.txt para deploy no Heroku
- Adiciona rota /resumo-execucao com detalhes da geração
- Adiciona rota POST /atualizar-dados para recarregar dados
- Habilita FLASK_SECRET_KEY e PORT via variáveis de ambiente
- Desabilita debug mode em produção
- Adiciona campo de busca/filtro no modal de exclusão por descrição
- Botão 'GERAR DOCUMENTO' inicia desabilitado até aplicar filtros
- Redireciona botão 'Ver' do histórico para /resumo-execucao
- Corrige formatação de lote e tipo_depósito na tabela
</commit_message>
<xml_diff>
--- a/data/historico/historico_documentos.xlsx
+++ b/data/historico/historico_documentos.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,17 +492,13 @@
       <c r="C2" t="n">
         <v>300</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>345346</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" s="1" t="n">
-        <v>46229.92942528935</v>
+        <v>46229.9451416088</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2436b635-d34f-4e71-9116-1291819daa38</t>
+          <t>7facf2f0-a5f3-4cf2-b7c5-b2f7d34d6da6</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -536,17 +532,13 @@
       <c r="C3" t="n">
         <v>300</v>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>345346</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" s="1" t="n">
-        <v>46229.92942528935</v>
+        <v>46229.9451416088</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2436b635-d34f-4e71-9116-1291819daa38</t>
+          <t>7facf2f0-a5f3-4cf2-b7c5-b2f7d34d6da6</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -580,17 +572,13 @@
       <c r="C4" t="n">
         <v>300</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>345346</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" s="1" t="n">
-        <v>46229.92942528935</v>
+        <v>46229.9451416088</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2436b635-d34f-4e71-9116-1291819daa38</t>
+          <t>7facf2f0-a5f3-4cf2-b7c5-b2f7d34d6da6</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -624,17 +612,13 @@
       <c r="C5" t="n">
         <v>300</v>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>345346</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" s="1" t="n">
-        <v>46229.92942528935</v>
+        <v>46229.9451416088</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2436b635-d34f-4e71-9116-1291819daa38</t>
+          <t>7facf2f0-a5f3-4cf2-b7c5-b2f7d34d6da6</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -668,17 +652,13 @@
       <c r="C6" t="n">
         <v>300</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>345346</t>
-        </is>
-      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" s="1" t="n">
-        <v>46229.92942528935</v>
+        <v>46229.9451416088</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2436b635-d34f-4e71-9116-1291819daa38</t>
+          <t>7facf2f0-a5f3-4cf2-b7c5-b2f7d34d6da6</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -700,6 +680,328 @@
       </c>
       <c r="L6" t="n">
         <v>1653323.6127568</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2000081.0</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2617402</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" s="1" t="n">
+        <v>46229.94527521631</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>b4e0b3e2-74d3-4597-abb9-48ce0cab50be</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>26969.7645</v>
+      </c>
+      <c r="J7" t="n">
+        <v>7</v>
+      </c>
+      <c r="K7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1255458.60284433</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>3000550.0</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2600004996</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" s="1" t="n">
+        <v>46229.94527521631</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>b4e0b3e2-74d3-4597-abb9-48ce0cab50be</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>10</v>
+      </c>
+      <c r="I8" t="n">
+        <v>157622.70799632</v>
+      </c>
+      <c r="J8" t="n">
+        <v>7</v>
+      </c>
+      <c r="K8" t="n">
+        <v>100</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1255458.60284433</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>3000550.0</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2600012494</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" s="1" t="n">
+        <v>46229.94527521631</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>b4e0b3e2-74d3-4597-abb9-48ce0cab50be</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>16</v>
+      </c>
+      <c r="I9" t="n">
+        <v>270211.82022797</v>
+      </c>
+      <c r="J9" t="n">
+        <v>7</v>
+      </c>
+      <c r="K9" t="n">
+        <v>100</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1255458.60284433</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>3000550.0</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2600016287</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" s="1" t="n">
+        <v>46229.94527521631</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>b4e0b3e2-74d3-4597-abb9-48ce0cab50be</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>12</v>
+      </c>
+      <c r="I10" t="n">
+        <v>202661.01</v>
+      </c>
+      <c r="J10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K10" t="n">
+        <v>100</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1255458.60284433</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>3000502.0</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2600015623</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" s="1" t="n">
+        <v>46229.94527521631</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>b4e0b3e2-74d3-4597-abb9-48ce0cab50be</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>39</v>
+      </c>
+      <c r="I11" t="n">
+        <v>237709.89737418</v>
+      </c>
+      <c r="J11" t="n">
+        <v>7</v>
+      </c>
+      <c r="K11" t="n">
+        <v>100</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1255458.60284433</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>3000550.0</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2600012581</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" s="1" t="n">
+        <v>46229.94527521631</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>b4e0b3e2-74d3-4597-abb9-48ce0cab50be</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>16</v>
+      </c>
+      <c r="I12" t="n">
+        <v>270211.84274586</v>
+      </c>
+      <c r="J12" t="n">
+        <v>7</v>
+      </c>
+      <c r="K12" t="n">
+        <v>100</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1255458.60284433</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3000550.0</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2600012493</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" s="1" t="n">
+        <v>46229.94527521631</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>b4e0b3e2-74d3-4597-abb9-48ce0cab50be</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" t="n">
+        <v>90071.56</v>
+      </c>
+      <c r="J13" t="n">
+        <v>7</v>
+      </c>
+      <c r="K13" t="n">
+        <v>100</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1255458.60284433</v>
       </c>
     </row>
   </sheetData>

</xml_diff>